<commit_message>
Added parts for new IC
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitRepos\golf-gps\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\gitRepos\golf-gps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13846F85-6011-4C3C-B3C7-95D0032E391F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD9F64D-7AE0-436C-A163-77E82B7F639B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Quantity</t>
   </si>
@@ -65,283 +65,13 @@
     <t>Vendor/LCSC PN</t>
   </si>
   <si>
-    <t>AE1</t>
+    <t>Total Part Count</t>
   </si>
   <si>
-    <t>BT1</t>
+    <t>Battery</t>
   </si>
   <si>
-    <t>BT2</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>FB1, FB2</t>
-  </si>
-  <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>J2</t>
-  </si>
-  <si>
-    <t>J3</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>R1</t>
-  </si>
-  <si>
-    <t>R3</t>
-  </si>
-  <si>
-    <t>C1, C5-8</t>
-  </si>
-  <si>
-    <t>C2, C4</t>
-  </si>
-  <si>
-    <t>C3, C9, C13-16, C19, C20, C23-26</t>
-  </si>
-  <si>
-    <t>C11, C17, C18</t>
-  </si>
-  <si>
-    <t>C21,22</t>
-  </si>
-  <si>
-    <t>C10, C12</t>
-  </si>
-  <si>
-    <t>D2, D3, D5</t>
-  </si>
-  <si>
-    <t>D4</t>
-  </si>
-  <si>
-    <t>R2, R6</t>
-  </si>
-  <si>
-    <t>R4</t>
-  </si>
-  <si>
-    <t>R5, R10-15</t>
-  </si>
-  <si>
-    <t>SW1</t>
-  </si>
-  <si>
-    <t>SW2-5</t>
-  </si>
-  <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>U4</t>
-  </si>
-  <si>
-    <t>Y1</t>
-  </si>
-  <si>
-    <t>STM32L432KCU6</t>
-  </si>
-  <si>
-    <t>C1337280</t>
-  </si>
-  <si>
-    <t>UFQFPN-32</t>
-  </si>
-  <si>
-    <t>STMicroelectronics</t>
-  </si>
-  <si>
-    <t>IC MCU 32BIT 256KB FLSH 32UFQFPN</t>
-  </si>
-  <si>
-    <t>USB4110-GF-A</t>
-  </si>
-  <si>
-    <t>2073-USB4110-GF-A-1-ND</t>
-  </si>
-  <si>
-    <t>GCT</t>
-  </si>
-  <si>
-    <t>CONN RCP USB2.0 TYP C 24P SMD RA</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>C3284251</t>
-  </si>
-  <si>
-    <t>RF ANT GNSS PATCH L1 12X12 SMD</t>
-  </si>
-  <si>
-    <t>TE Connectivity Linx</t>
-  </si>
-  <si>
-    <t>ANT-GNSSCP-SM12L1</t>
-  </si>
-  <si>
-    <t>CR2032 Coin Cell Battery Holder</t>
-  </si>
-  <si>
-    <t>PRTR5V0U2X</t>
-  </si>
-  <si>
-    <t>C2827688</t>
-  </si>
-  <si>
-    <t>SOT-143</t>
-  </si>
-  <si>
-    <t>TECH PUBLIC</t>
-  </si>
-  <si>
-    <t>TVS DIODE 5.5VWM SOT143B</t>
-  </si>
-  <si>
-    <t>ETG</t>
-  </si>
-  <si>
-    <t>C424093</t>
-  </si>
-  <si>
-    <t>MCP73831T-2ACI/OT</t>
-  </si>
-  <si>
-    <t>SOT-23-5</t>
-  </si>
-  <si>
-    <t>Microchip Tech</t>
-  </si>
-  <si>
-    <t>IC BATT CNTL LI-ION 1CEL SOT23-5</t>
-  </si>
-  <si>
-    <t>Connector for 1.8" TFT LCD from ETG</t>
-  </si>
-  <si>
-    <t>CONN HEADER VERT 8POS 2.54MM</t>
-  </si>
-  <si>
-    <t>P=2.54mm</t>
-  </si>
-  <si>
-    <t>NEO-M9N</t>
-  </si>
-  <si>
-    <t>C5119087</t>
-  </si>
-  <si>
-    <t>M9 STANDARD PRECISION GNSS MOD</t>
-  </si>
-  <si>
-    <t>U-BLOX</t>
-  </si>
-  <si>
-    <t>SMD-24P</t>
-  </si>
-  <si>
-    <t>X206032768KGB2SC</t>
-  </si>
-  <si>
-    <t>C2236</t>
-  </si>
-  <si>
-    <t>DT-26</t>
-  </si>
-  <si>
-    <t>YXC Crystal Oscillators</t>
-  </si>
-  <si>
-    <t>CRYSTAL 32.7680KHZ 12.5PF TH</t>
-  </si>
-  <si>
-    <t>~1000mAh Lithium Ion Battery</t>
-  </si>
-  <si>
-    <t>BAT54C</t>
-  </si>
-  <si>
-    <t>C2135</t>
-  </si>
-  <si>
-    <t>SOT-23-3</t>
-  </si>
-  <si>
-    <t>Jiangsu Changjing Electronics Technology</t>
-  </si>
-  <si>
-    <t>DIODE ARR SCHOTT 30V 200MA SOT23</t>
-  </si>
-  <si>
-    <t>Bel Fuse Inc.</t>
-  </si>
-  <si>
-    <t>0ZCG0050AF2C</t>
-  </si>
-  <si>
-    <t>C3762102</t>
-  </si>
-  <si>
-    <t>PTC RESET FUSE 30V 500MA 1812</t>
-  </si>
-  <si>
-    <t>EG1218</t>
-  </si>
-  <si>
-    <t>P=2.50mm</t>
-  </si>
-  <si>
-    <t>E-Switch</t>
-  </si>
-  <si>
-    <t>SWITCH SLIDE SPDT 200MA 30V</t>
-  </si>
-  <si>
-    <t>6mm</t>
-  </si>
-  <si>
-    <t>SPDT PUSH BUTTON</t>
-  </si>
-  <si>
-    <t>C15516</t>
-  </si>
-  <si>
-    <t>TPS63031DSKR</t>
-  </si>
-  <si>
-    <t>IC REG BUCK BST 3.3V 900MA 10SON</t>
-  </si>
-  <si>
-    <t>Texas Instruments</t>
-  </si>
-  <si>
-    <t>10-WFDFN</t>
-  </si>
-  <si>
-    <t>Total Part Count</t>
+    <t xml:space="preserve">https://www.amazon.com/GYMIN-Rechargeable-Replacement-Steelseries-Wireless/dp/B0CRP2G3XN/ref=sr_1_6?crid=2SVHWDACPRGY&amp;dib=eyJ2IjoiMSJ9.tzaNrZ0FfVoEqsyG3x4WrCyq7T4EKo4Qlhkjs9kn6gR9N-SfnEHgcjt1sQaR1B-DQQgdjWPGQijsYK-rLaIoR1atM1zc9Fbt5MXDe6q1it4jjVHUb1ypACpoqtZxKN88-puW4kw9D4ij-7mQ85bko5kuYfOtpXuo1ExsoAl55K3fhH_tOdwWrD3JPgCigNzfQoW4ZhWttBjdh5Mt6B9sYDQwu3ZMzNouTObtmxDF3VaHZIuReUeWcgJoU7smvoZ62EmG6MirSUX7Gn9CPOnB8JPDaCa-ZZYnLyllHSiYVsg.DXLszwYu1Al4qQexpbaSAGerxHcQQeEKezpAKR6sRPI&amp;dib_tag=se&amp;keywords=3.7v+lithium+ion+battery+with+thermistor&amp;qid=1759337770&amp;sprefix=lithium+ion+battery+with+thermi%2Caps%2C102&amp;sr=8-6 </t>
   </si>
 </sst>
 </file>
@@ -1075,19 +805,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="20.21875" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="37.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="36.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="36.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1113,69 +843,39 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="12">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>50</v>
-      </c>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="12"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="12">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="12"/>
+      <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="12">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="12"/>
+      <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="7"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="12">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="12"/>
+      <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="2"/>
@@ -1183,13 +883,9 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="12">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
-      </c>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="2"/>
       <c r="C6" s="7"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1197,13 +893,9 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="12">
-        <v>12</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>24</v>
-      </c>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="12"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -1211,13 +903,9 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="12">
-        <v>3</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>25</v>
-      </c>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="12"/>
+      <c r="B8" s="2"/>
       <c r="C8" s="6"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -1225,13 +913,9 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="12">
-        <v>2</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>27</v>
-      </c>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="12"/>
+      <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="7"/>
       <c r="E9" s="2"/>
@@ -1239,13 +923,9 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="12">
-        <v>2</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>26</v>
-      </c>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="12"/>
+      <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -1253,37 +933,19 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="12">
-        <v>1</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>59</v>
-      </c>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="12"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="12">
-        <v>3</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>28</v>
-      </c>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="12"/>
+      <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -1291,61 +953,29 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="12">
-        <v>1</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>84</v>
-      </c>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="12"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
       <c r="H13" s="8"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="12">
-        <v>1</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E14" s="9">
-        <v>1812</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>88</v>
-      </c>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="12"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="12">
-        <v>2</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>13</v>
-      </c>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="12"/>
+      <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -1353,13 +983,9 @@
       <c r="G15" s="2"/>
       <c r="H15" s="8"/>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="12">
-        <v>1</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>14</v>
-      </c>
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12"/>
+      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -1367,33 +993,19 @@
       <c r="G16" s="2"/>
       <c r="H16" s="8"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="12">
-        <v>1</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>15</v>
-      </c>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="12"/>
+      <c r="B17" s="2"/>
       <c r="C17" s="5"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="4" t="s">
-        <v>68</v>
-      </c>
+      <c r="E17" s="4"/>
       <c r="F17" s="5"/>
-      <c r="G17" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="12">
-        <v>1</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="12"/>
+      <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
@@ -1401,13 +1013,9 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="12">
-        <v>1</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>17</v>
-      </c>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="12"/>
+      <c r="B19" s="2"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="2"/>
@@ -1415,13 +1023,9 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="12">
-        <v>1</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>18</v>
-      </c>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="12"/>
+      <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -1429,37 +1033,19 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="12">
-        <v>1</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>46</v>
-      </c>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="12"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="12">
-        <v>1</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="12"/>
+      <c r="B22" s="2"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
       <c r="E22" s="2"/>
@@ -1467,13 +1053,9 @@
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="12">
-        <v>2</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>30</v>
-      </c>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="12"/>
+      <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -1481,13 +1063,9 @@
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="12">
-        <v>1</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>21</v>
-      </c>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="12"/>
+      <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1495,13 +1073,9 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="12">
-        <v>1</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>31</v>
-      </c>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="12"/>
+      <c r="B25" s="2"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="2"/>
@@ -1509,13 +1083,9 @@
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="12">
-        <v>7</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>32</v>
-      </c>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="12"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="5"/>
       <c r="E26" s="2"/>
@@ -1523,171 +1093,81 @@
       <c r="G26" s="2"/>
       <c r="H26" s="8"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="12">
-        <v>1</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>89</v>
-      </c>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="12"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="12">
-        <v>4</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>34</v>
-      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="12"/>
+      <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="2" t="s">
-        <v>93</v>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="10"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="12"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="12"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2" t="s">
+        <v>9</v>
       </c>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2" t="s">
-        <v>94</v>
+      <c r="H30" s="2" t="s">
+        <v>10</v>
       </c>
-      <c r="H28" s="10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="12">
-        <v>1</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="12">
-        <v>1</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="12">
-        <v>1</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>44</v>
-      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="12"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="12">
-        <v>1</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>71</v>
-      </c>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="12"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="12">
-        <v>1</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>78</v>
-      </c>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="12"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="11"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1697,7 +1177,7 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="11"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1707,7 +1187,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="11"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1717,13 +1197,13 @@
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="14">
         <f>SUM(A2:A36)</f>
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>100</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1731,7 +1211,7 @@
   <pageMargins left="0.67965686274509796" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="59" orientation="landscape" r:id="rId1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;"-,Bold"&amp;14Golf GPS BOM&amp;RRev 0</oddHeader>
+    <oddHeader>&amp;C&amp;"-,Bold"&amp;14Golf GPS BOM&amp;RRev 1</oddHeader>
   </headerFooter>
   <tableParts count="1">
     <tablePart r:id="rId2"/>

</xml_diff>

<commit_message>
Started BOM, changed micrsoSD card slot and some other footprint. Will need to update layout.
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\gitRepos\golf-gps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD9F64D-7AE0-436C-A163-77E82B7F639B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5038BFDD-FF1E-46AA-A52B-1E66A823809A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">BOM!$A$1:$H$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">BOM!$A$1:$H$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="79">
   <si>
     <t>Quantity</t>
   </si>
@@ -62,16 +62,232 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Vendor/LCSC PN</t>
-  </si>
-  <si>
     <t>Total Part Count</t>
   </si>
   <si>
-    <t>Battery</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.amazon.com/GYMIN-Rechargeable-Replacement-Steelseries-Wireless/dp/B0CRP2G3XN/ref=sr_1_6?crid=2SVHWDACPRGY&amp;dib=eyJ2IjoiMSJ9.tzaNrZ0FfVoEqsyG3x4WrCyq7T4EKo4Qlhkjs9kn6gR9N-SfnEHgcjt1sQaR1B-DQQgdjWPGQijsYK-rLaIoR1atM1zc9Fbt5MXDe6q1it4jjVHUb1ypACpoqtZxKN88-puW4kw9D4ij-7mQ85bko5kuYfOtpXuo1ExsoAl55K3fhH_tOdwWrD3JPgCigNzfQoW4ZhWttBjdh5Mt6B9sYDQwu3ZMzNouTObtmxDF3VaHZIuReUeWcgJoU7smvoZ62EmG6MirSUX7Gn9CPOnB8JPDaCa-ZZYnLyllHSiYVsg.DXLszwYu1Al4qQexpbaSAGerxHcQQeEKezpAKR6sRPI&amp;dib_tag=se&amp;keywords=3.7v+lithium+ion+battery+with+thermistor&amp;qid=1759337770&amp;sprefix=lithium+ion+battery+with+thermi%2Caps%2C102&amp;sr=8-6 </t>
+  </si>
+  <si>
+    <t>AE1</t>
+  </si>
+  <si>
+    <t>BT1</t>
+  </si>
+  <si>
+    <t>BT2</t>
+  </si>
+  <si>
+    <t>C1, C8, C10, C12, C14, C16, C17, C22, C23</t>
+  </si>
+  <si>
+    <t>C0603</t>
+  </si>
+  <si>
+    <t>C2-C7, C9</t>
+  </si>
+  <si>
+    <t>C11, C19, C25</t>
+  </si>
+  <si>
+    <t>C13, C15</t>
+  </si>
+  <si>
+    <t>C18, C24</t>
+  </si>
+  <si>
+    <t>C20, C21</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2-D4</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>J1-J3</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>J5</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>DNP. Use 0603 0 Ohm resistor</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>R1, R4, R7, R12-R14, R16-R21</t>
+  </si>
+  <si>
+    <t>R2, R3</t>
+  </si>
+  <si>
+    <t>R5</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>R8-R11, R15</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>SW2-SW5</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>TP1-TP11</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>U4</t>
+  </si>
+  <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>U6</t>
+  </si>
+  <si>
+    <t>U7</t>
+  </si>
+  <si>
+    <t>U8</t>
+  </si>
+  <si>
+    <t>Y1</t>
+  </si>
+  <si>
+    <t>Vendor PN</t>
+  </si>
+  <si>
+    <t>C0805</t>
+  </si>
+  <si>
+    <t>1727-3884-1-ND</t>
+  </si>
+  <si>
+    <t>PRTR5V0U2X,215</t>
+  </si>
+  <si>
+    <t>Nexperia USA Inc.</t>
+  </si>
+  <si>
+    <t>SOT-143B</t>
+  </si>
+  <si>
+    <t>D0805</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5.5VWM SOT143B</t>
+  </si>
+  <si>
+    <t>LED RED CLEAR SMD 0805</t>
+  </si>
+  <si>
+    <t>LTST-C170CKT</t>
+  </si>
+  <si>
+    <t>Lite-On Inc.</t>
+  </si>
+  <si>
+    <t>ETG Stock</t>
+  </si>
+  <si>
+    <t>LED GREEN CLEAR SMD 0805</t>
+  </si>
+  <si>
+    <t>160-1179-1-ND</t>
+  </si>
+  <si>
+    <t>LTST-C170GKT</t>
+  </si>
+  <si>
+    <t>4878-BAT54CCT-ND</t>
+  </si>
+  <si>
+    <t>Diotec Semiconductor</t>
+  </si>
+  <si>
+    <t>DIODE ARR SCHOTT 30V 200MA SOT23</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>BAT54C</t>
+  </si>
+  <si>
+    <t>D5, D7</t>
+  </si>
+  <si>
+    <t>0ZCJ0100FF2E</t>
+  </si>
+  <si>
+    <t>Bel Fuse Inc.</t>
+  </si>
+  <si>
+    <t>5923-0ZCJ0100FF2ECT-ND</t>
+  </si>
+  <si>
+    <t>PTC RESET FUSE 6V 1A 1206</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ETG Stock </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(double check)</t>
+    </r>
+  </si>
+  <si>
+    <t>WM6357CT-ND</t>
+  </si>
+  <si>
+    <t>Molex</t>
+  </si>
+  <si>
+    <t>CONN MICRO SD CARD R/A SMD</t>
+  </si>
+  <si>
+    <t>1040310811</t>
   </si>
 </sst>
 </file>
@@ -156,7 +372,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -179,12 +395,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="9"/>
+      </left>
+      <right style="thin">
+        <color theme="9"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="9"/>
+      </left>
+      <right style="thin">
+        <color theme="9"/>
+      </right>
+      <top style="thin">
+        <color theme="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </left>
+      <right style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -193,7 +450,6 @@
     <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -204,28 +460,176 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -240,7 +644,7 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color theme="9"/>
@@ -271,97 +675,7 @@
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color theme="9"/>
         </left>
@@ -516,8 +830,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:H36" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H36" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:I39" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I39" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -526,16 +840,18 @@
     <filterColumn colId="5" hiddenButton="1"/>
     <filterColumn colId="6" hiddenButton="1"/>
     <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor/LCSC PN" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{830C4442-5AB3-43AC-A769-0794297CBDA1}" name="Package" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{108683D9-DF72-46B8-9EFA-4A90CB8F9C65}" name="Manufacturer" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{0288C8FE-25DB-42B5-9EE0-77B481F28BD2}" name="Description" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="0"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -804,20 +1120,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="36.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -825,386 +1142,685 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="I1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="I2" s="10"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="16">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="7"/>
+      <c r="I3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="16">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="6"/>
       <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="12"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="16">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="16">
+        <v>7</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="12"/>
+      <c r="D6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="12"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="16">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="16">
+        <v>2</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="12"/>
+      <c r="D8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="7"/>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="16">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="6"/>
       <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="16">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="16">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="16">
+        <v>3</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>59</v>
+      </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
+        <v>2</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="16">
+        <v>1</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="8"/>
-    </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16">
+        <v>1</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" s="7"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="16">
+        <v>3</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="8"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I16" s="2"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="16">
+        <v>1</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="16">
+        <v>1</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
       <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="16">
+        <v>1</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="16">
+        <v>1</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="16">
+        <v>1</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
       <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="12"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="I21" s="2"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="16">
+        <v>1</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="I22" s="2"/>
+    </row>
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="16">
+        <v>12</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="I23" s="2"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="16">
+        <v>2</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
       <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
+      <c r="I24" s="2"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="16">
+        <v>1</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="12"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="5"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="2"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="16">
+        <v>1</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
-      <c r="H26" s="8"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="16">
+        <v>5</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="12"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="2"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="16">
+        <v>1</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
-      <c r="H28" s="10"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="12"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>4</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="12"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="16">
+        <v>11</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
-      <c r="G30" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="12"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="5"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="16">
+        <v>1</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="12"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
+      <c r="I31" s="2"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="16">
+        <v>1</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="12"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
+      <c r="I32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="16">
+        <v>1</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
+      <c r="I33" s="2"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="16">
+        <v>1</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="11"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="I34" s="2"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="16">
+        <v>1</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="11"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="14">
-        <f>SUM(A2:A36)</f>
-        <v>0</v>
-      </c>
-      <c r="B37" s="13" t="s">
-        <v>8</v>
-      </c>
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="17">
+        <v>1</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="17">
+        <v>1</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="17">
+        <v>1</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="11"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="17">
+        <v>1</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="11"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="15">
+        <f>SUM(A2:A39)</f>
+        <v>91</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Moved some things around, revised regulator layout
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\gitRepos\golf-gps\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bjkuh\Projects\gitRepos\golf-gps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5038BFDD-FF1E-46AA-A52B-1E66A823809A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4622297A-BD68-495C-B339-EA18871F265E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -470,22 +470,22 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -498,6 +498,96 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -517,6 +607,70 @@
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color theme="9"/>
@@ -568,11 +722,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -585,7 +735,7 @@
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color theme="9"/>
         </left>
@@ -595,9 +745,9 @@
         <top style="thin">
           <color theme="9"/>
         </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -615,156 +765,6 @@
       </font>
       <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color theme="9"/>
@@ -843,15 +843,15 @@
     <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Lots of layout progress, changed some references (need to update BOM)
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bjkuh\Projects\gitRepos\golf-gps\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\golf-gps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4622297A-BD68-495C-B339-EA18871F265E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E46221-5B72-4825-9D27-95804757E5E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">BOM!$A$1:$H$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">BOM!$A$1:$H$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="89">
   <si>
     <t>Quantity</t>
   </si>
@@ -77,27 +77,15 @@
     <t>BT2</t>
   </si>
   <si>
-    <t>C1, C8, C10, C12, C14, C16, C17, C22, C23</t>
-  </si>
-  <si>
     <t>C0603</t>
   </si>
   <si>
     <t>C2-C7, C9</t>
   </si>
   <si>
-    <t>C11, C19, C25</t>
-  </si>
-  <si>
     <t>C13, C15</t>
   </si>
   <si>
-    <t>C18, C24</t>
-  </si>
-  <si>
-    <t>C20, C21</t>
-  </si>
-  <si>
     <t>D1</t>
   </si>
   <si>
@@ -110,15 +98,6 @@
     <t>F1</t>
   </si>
   <si>
-    <t>J1-J3</t>
-  </si>
-  <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>J5</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -134,21 +113,9 @@
     <t>Q1</t>
   </si>
   <si>
-    <t>R1, R4, R7, R12-R14, R16-R21</t>
-  </si>
-  <si>
     <t>R2, R3</t>
   </si>
   <si>
-    <t>R5</t>
-  </si>
-  <si>
-    <t>R6</t>
-  </si>
-  <si>
-    <t>R8-R11, R15</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -180,9 +147,6 @@
   </si>
   <si>
     <t>U7</t>
-  </si>
-  <si>
-    <t>U8</t>
   </si>
   <si>
     <t>Y1</t>
@@ -288,6 +252,72 @@
   </si>
   <si>
     <t>1040310811</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>B0CRP2G3XN</t>
+  </si>
+  <si>
+    <t>GYMIN</t>
+  </si>
+  <si>
+    <t>1500mAh LiPo Battery</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>CONN RCP USB2.0 TYP C 24P SMD RA</t>
+  </si>
+  <si>
+    <t>USB4105-GF-A</t>
+  </si>
+  <si>
+    <t>GCT</t>
+  </si>
+  <si>
+    <t>2073-USB4105-GF-ACT-ND</t>
+  </si>
+  <si>
+    <t>C1, C8, C10, C12, C14, C16, C17, C20, C21</t>
+  </si>
+  <si>
+    <t>Value TBD</t>
+  </si>
+  <si>
+    <t>C11, C23</t>
+  </si>
+  <si>
+    <t>C22</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>J8</t>
+  </si>
+  <si>
+    <t>J3-J5</t>
+  </si>
+  <si>
+    <t>J6</t>
+  </si>
+  <si>
+    <t>J7</t>
+  </si>
+  <si>
+    <t>R1, R4, R8, R13-R15, R17-R22</t>
+  </si>
+  <si>
+    <t>R5, R6</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>R9-R12, R16</t>
   </si>
 </sst>
 </file>
@@ -830,8 +860,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:I39" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I39" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:I41" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I41" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1120,7 +1150,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1154,13 +1184,13 @@
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1185,12 +1215,20 @@
       <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="4" t="s">
+        <v>70</v>
+      </c>
       <c r="D3" s="4"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
@@ -1215,11 +1253,11 @@
         <v>9</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -1232,11 +1270,11 @@
         <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="2" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -1249,11 +1287,11 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -1266,16 +1304,18 @@
         <v>2</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1283,11 +1323,11 @@
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>17</v>
+        <v>79</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="13"/>
@@ -1299,13 +1339,9 @@
       <c r="A10" s="16">
         <v>2</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>18</v>
-      </c>
+      <c r="B10" s="4"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1317,22 +1353,22 @@
         <v>1</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -1342,23 +1378,23 @@
         <v>3</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="I12" s="2"/>
     </row>
@@ -1367,25 +1403,25 @@
         <v>2</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -1394,22 +1430,22 @@
         <v>1</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -1419,79 +1455,77 @@
         <v>1</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="2" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="H15" s="7"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2" t="s">
-        <v>60</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="14"/>
+      <c r="E16" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H16" s="7"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="16">
         <v>1</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>74</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="7"/>
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1499,12 +1533,12 @@
         <v>1</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
+        <v>83</v>
+      </c>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="F19" s="11"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -1514,15 +1548,15 @@
         <v>1</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+        <v>84</v>
+      </c>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="I20" s="2"/>
     </row>
@@ -1531,14 +1565,24 @@
         <v>1</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="I21" s="2"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1546,7 +1590,7 @@
         <v>1</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -1556,27 +1600,29 @@
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="16">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="I23" s="2"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
@@ -1591,22 +1637,22 @@
         <v>1</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="7"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
       <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="16">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -1618,17 +1664,17 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="16">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="8"/>
+        <v>24</v>
+      </c>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="2"/>
       <c r="I27" s="2"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1636,22 +1682,22 @@
         <v>1</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="7"/>
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -1663,17 +1709,17 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="16">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="8"/>
       <c r="I30" s="2"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -1681,7 +1727,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
@@ -1693,10 +1739,10 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -1708,16 +1754,16 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="16">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
+      <c r="G33" s="4"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
     </row>
@@ -1726,7 +1772,7 @@
         <v>1</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -1741,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -1749,51 +1795,51 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="11"/>
+      <c r="I35" s="2"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="17">
-        <v>1</v>
-      </c>
-      <c r="B36" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
+      <c r="A36" s="16">
+        <v>1</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="17">
-        <v>1</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
+      <c r="A37" s="16">
+        <v>1</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="17">
-        <v>1</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
+      <c r="A38" s="16">
+        <v>1</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
       <c r="I38" s="11"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -1801,7 +1847,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C39" s="14"/>
       <c r="D39" s="14"/>
@@ -1812,15 +1858,45 @@
       <c r="I39" s="11"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="15">
-        <f>SUM(A2:A39)</f>
-        <v>91</v>
-      </c>
-      <c r="B40" s="9" t="s">
+      <c r="A40" s="17">
+        <v>1</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="17">
+        <v>1</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="15">
+        <f>SUM(A2:A41)</f>
+        <v>93</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Worked on BOM List
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\golf-gps\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1eb1c9bb38a56ae9/Documents/CollegeInformation/2025-2026/EE333/golf-gps/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E46221-5B72-4825-9D27-95804757E5E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="13_ncr:1_{C2E46221-5B72-4825-9D27-95804757E5E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9943607C-E0A9-496C-9C29-41D18440A4C6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-9610" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">BOM!$A$1:$H$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">BOM!$A$1:$H$31</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="222">
   <si>
     <t>Quantity</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>DNP. Use 0603 0 Ohm resistor</t>
-  </si>
-  <si>
-    <t>P1</t>
   </si>
   <si>
     <t>Q1</t>
@@ -319,12 +316,414 @@
   <si>
     <t>R9-R12, R16</t>
   </si>
+  <si>
+    <t>RF ANT 1.575/1.602GHZ CER PATCH</t>
+  </si>
+  <si>
+    <t>SGGP.25.2.A.02</t>
+  </si>
+  <si>
+    <t>Taoglas Limited</t>
+  </si>
+  <si>
+    <t>931-1450-1-ND</t>
+  </si>
+  <si>
+    <t>RF ANTENNA GLONASS, GPS Ceramic Patch Solder Surface Mount</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/taoglas-limited/SGGP-25-2-A-02/6362788?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=17922795960&amp;gbraid=0AAAAADrbLlgMcI_xxgM1XnWlukN8LfDyD&amp;gclid=Cj0KCQjwl5jHBhDHARIsAB0YqjwtykcaCqflOK956I59n-BT9VoB2bK0Yaz9wxJRDuOLV2NKlyDRbr8aAiUgEALw_wcB</t>
+  </si>
+  <si>
+    <t>Battery Retainer Coin, 20.0mm 1 Cell SMD (SMT) Tab</t>
+  </si>
+  <si>
+    <t>3002</t>
+  </si>
+  <si>
+    <t>Keystone Electronics</t>
+  </si>
+  <si>
+    <t>36-3002-ND</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 50V X7R 0603</t>
+  </si>
+  <si>
+    <t>CL10B104KB8NNNC</t>
+  </si>
+  <si>
+    <t>Samsung Electro-Mechanics</t>
+  </si>
+  <si>
+    <t>1276-1000-1-ND</t>
+  </si>
+  <si>
+    <t>CAP CER 10UF 16V X5R 0805</t>
+  </si>
+  <si>
+    <t>CL21A106KOQNNNG</t>
+  </si>
+  <si>
+    <t>1276-6455-1-ND</t>
+  </si>
+  <si>
+    <t>160-1176-1-ND</t>
+  </si>
+  <si>
+    <t>Diode Array 1 Pair Common Cathode 30 V 200mA Surface Mount TO-236-3, SC-59, SOT-23-3</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/diotec-semiconductor/bat54c/13163831</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 kOhms ±1% 0.125W, 1/8W </t>
+  </si>
+  <si>
+    <t>R0603</t>
+  </si>
+  <si>
+    <t>RNCP0603FTD10K0</t>
+  </si>
+  <si>
+    <t>Stackpole Electronics Inc</t>
+  </si>
+  <si>
+    <t>RNCP0603FTD10K0CT-ND</t>
+  </si>
+  <si>
+    <t>CL10A105KA8NNNC</t>
+  </si>
+  <si>
+    <t>1276-1102-1-ND</t>
+  </si>
+  <si>
+    <t>CAP CER 1UF 25V X5R 0603</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>CL10A225KO8NNNC</t>
+  </si>
+  <si>
+    <t>1276-1040-1-ND</t>
+  </si>
+  <si>
+    <t>2.2 µF ±10% 16V Ceramic Capacitor X5R 0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>CAP CER 2.2UF 16V X5R 0603</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10A225KO8NNNC/3886698</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/gct/usb4105-gf-a-120/14559037?_gl=1*8ga6od*_up*MQ..*_gs*MQ..&amp;gclid=Cj0KCQjwgKjHBhChARIsAPJR3xcbwCelwdcfWysaQJ6lGrexOVJoh9QxdhYzJnLbXn23lASGFgIhokAaAg0aEALw_wcB&amp;gclsrc=aw.ds&amp;gbraid=0AAAAADrbLli0aKyISK_R9nHbxT6VDbqY_</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/molex/1040310811/2370379?s=N4IgTCBcDaIOoFkBsBmArAdgMIBUC0AcgCIgC6AvkA</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Coilcraft/LPS3010-152MRC?qs=QQJxVsr8EGasSZ6gWEcu2Q%3D%3D</t>
+  </si>
+  <si>
+    <t>MOUSER</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Coilcraft</t>
+  </si>
+  <si>
+    <t>994-LPS3010-152MRC</t>
+  </si>
+  <si>
+    <t>LPS3010-152MRC</t>
+  </si>
+  <si>
+    <t>Power Inductors - SMD 1.5uH Shld 20% 120mOhms AECQ2</t>
+  </si>
+  <si>
+    <t>LPS3010</t>
+  </si>
+  <si>
+    <t>MOSFET P-CH 20V 4.2A SOT23</t>
+  </si>
+  <si>
+    <t>TO-236-3, SC-59, SOT-23-3</t>
+  </si>
+  <si>
+    <t>DMG2305UX-7</t>
+  </si>
+  <si>
+    <t>Diodes Incorporated</t>
+  </si>
+  <si>
+    <t>P-Channel 20 V 4.2A (Ta) 1.4W (Ta) Surface Mount SOT-23-3</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/diodes-incorporated/dmg2305ux-7/4340667</t>
+  </si>
+  <si>
+    <t>311-27GRCT-ND</t>
+  </si>
+  <si>
+    <t>YAGEO</t>
+  </si>
+  <si>
+    <t>RC0603JR-0727RL</t>
+  </si>
+  <si>
+    <t>27 Ohms ±5% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603JR-0727RL/726751</t>
+  </si>
+  <si>
+    <t>RES 27 OHM 5% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-075K1L</t>
+  </si>
+  <si>
+    <t>311-5.10KHRCT-ND</t>
+  </si>
+  <si>
+    <t>RES 5.1K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>5.1 kOhms ±1% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-075K1L/727268</t>
+  </si>
+  <si>
+    <t>RC0603JR-071K3L</t>
+  </si>
+  <si>
+    <t>311-1.3KGRCT-ND</t>
+  </si>
+  <si>
+    <t>1.3 kOhms ±5% 0.1W, 1/10W Chip Resistor 0603 (1608 Metric) Moisture Resistant Thick Film</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603JR-071K3L/726686</t>
+  </si>
+  <si>
+    <t>RES 1.3K OHM 5% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RES 1K OHM 1% 1/8W 0603</t>
+  </si>
+  <si>
+    <t>RNCP0603FTD1K00</t>
+  </si>
+  <si>
+    <t>RNCP0603FTD1K00CT-ND</t>
+  </si>
+  <si>
+    <t>450301014042</t>
+  </si>
+  <si>
+    <t>Würth Elektronik</t>
+  </si>
+  <si>
+    <t>SWITCH SLIDE SPDT 500MA 12V</t>
+  </si>
+  <si>
+    <t>Slide Switch SPDT Through Hole</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/w%C3%BCrth-elektronik/450301014042/5209104</t>
+  </si>
+  <si>
+    <t>450301014042-ND</t>
+  </si>
+  <si>
+    <t>WS-SLTV</t>
+  </si>
+  <si>
+    <t>TS02-66-43-BK-160-LCR-D</t>
+  </si>
+  <si>
+    <t>2223-TS02-66-43-BK-160-LCR-D-ND</t>
+  </si>
+  <si>
+    <t>Same Sky (Formerly CUI Devices)</t>
+  </si>
+  <si>
+    <t>Tactile Switch SPST-NO Top Actuated Through Hole</t>
+  </si>
+  <si>
+    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
+  </si>
+  <si>
+    <t>TS02</t>
+  </si>
+  <si>
+    <t>768-1178-1-ND</t>
+  </si>
+  <si>
+    <t>USB Bridge, USB to UART USB 2.0 UART Interface 12-DFN (3x3)</t>
+  </si>
+  <si>
+    <t>FTDI, Future Technology Devices International Ltd</t>
+  </si>
+  <si>
+    <t>FT234XD-R</t>
+  </si>
+  <si>
+    <t>IC USB SERIAL BASIC UART 12DFN</t>
+  </si>
+  <si>
+    <t>12-VFDFN Exposed Pad</t>
+  </si>
+  <si>
+    <t>MCP73871-1AAI/ML-ND</t>
+  </si>
+  <si>
+    <t>Microchip Technology</t>
+  </si>
+  <si>
+    <t>IC BATT CHG LI-ION 1CELL 20QFN</t>
+  </si>
+  <si>
+    <t>Charger IC Lithium Ion/Polymer 20-QFN (4x4)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/microchip-technology/mcp73871-1aai-ml/7928179</t>
+  </si>
+  <si>
+    <t>20-VFQFN Exposed Pad</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/ftdi-future-technology-devices-international-ltd/FT234XD-R/3904921?s=N4IgTCBcDaIOwDYAcBaAjGuq0oHIBEQBdAXyA</t>
+  </si>
+  <si>
+    <t>TPS63031DSKR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>296-39461-1-ND</t>
+  </si>
+  <si>
+    <t>IC REG BUCK BST 3.3V 900MA 10SON</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TPS63031DSKR/2048021?s=N4IgTCBcDaICoAUDKA2AzABjQRgCJIGkAlEAXQF8g</t>
+  </si>
+  <si>
+    <t>Buck-Boost Switching Regulator IC Positive Fixed 3.3V 1 Output 900mA (Switch) 10-WFDFN Exposed Pad</t>
+  </si>
+  <si>
+    <t>10-WFDFN Exposed Pad</t>
+  </si>
+  <si>
+    <t>ESP32-C3-WROOM-02-H4</t>
+  </si>
+  <si>
+    <t>Espressif Systems</t>
+  </si>
+  <si>
+    <t>1965-ESP32-C3-WROOM-02-H4CT-ND</t>
+  </si>
+  <si>
+    <t>Bluetooth, WiFi 802.11b/g/n, Bluetooth v5.0 Transceiver Module 2.4GHz PCB Trace Surface Mount</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/espressif-systems/esp32-c3-wroom-02-h4/14553033</t>
+  </si>
+  <si>
+    <t>32-SMD Module</t>
+  </si>
+  <si>
+    <t>672-NEO-M9N-00BCT-ND</t>
+  </si>
+  <si>
+    <t>NEO-M9N-00B</t>
+  </si>
+  <si>
+    <t>u-blox</t>
+  </si>
+  <si>
+    <t>M9 RF Receiver BeiDou, Galileo, GLONASS, GNSS, GPS -167dBm Module</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/u-blox/neo-m9n-00b/12149174</t>
+  </si>
+  <si>
+    <t>M9 STANDARD PRECISION GNSS MOD</t>
+  </si>
+  <si>
+    <t>24-SMD Module</t>
+  </si>
+  <si>
+    <t>296-BQ27427YZFRCT-ND</t>
+  </si>
+  <si>
+    <t>Battery Fuel Gauge IC Lithium Ion 9-DSBGA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/BQ27427YZFR/17748369</t>
+  </si>
+  <si>
+    <t>BQ27427YZFR</t>
+  </si>
+  <si>
+    <t>SINGLE-CELL BATTERY FUEL GAUGE W</t>
+  </si>
+  <si>
+    <t>9-DSBGA</t>
+  </si>
+  <si>
+    <t>Sensirion AG</t>
+  </si>
+  <si>
+    <t>SHT30-DIS-B2.5KS</t>
+  </si>
+  <si>
+    <t>1649-1009-1-ND</t>
+  </si>
+  <si>
+    <t>Humidity, Temperature 0 ~ 100% RH I2C ±2% RH 8 s Surface Mount</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/sensirion-ag/SHT30-DIS-B2-5KS/5872250</t>
+  </si>
+  <si>
+    <t>SENSOR HUMID/TEMP 5V I2C 2% SMD</t>
+  </si>
+  <si>
+    <t>8-VFDFN Exposed Pad</t>
+  </si>
+  <si>
+    <t>ABS07-32.768KHZ-T</t>
+  </si>
+  <si>
+    <t>Abracon LLC</t>
+  </si>
+  <si>
+    <t>CRYSTAL 32.7680KHZ 12.5PF SMD</t>
+  </si>
+  <si>
+    <t>32.768 kHz ±20ppm Crystal 12.5pF 70 kOhms 2-SMD, No Lead</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/abracon-llc/ABS07-32-768KHZ-T/1236858</t>
+  </si>
+  <si>
+    <t>2-SMD (3.2x1.5)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,8 +780,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF444444"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -391,18 +815,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -466,18 +902,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -522,12 +966,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -860,8 +1364,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:I41" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I41" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:J40" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J40" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -871,17 +1375,19 @@
     <filterColumn colId="6" hiddenButton="1"/>
     <filterColumn colId="7" hiddenButton="1"/>
     <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="0"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{04A78D46-042E-424E-B45C-FB7EBC025E60}" name="Column1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1150,21 +1656,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J41"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" customWidth="1"/>
-    <col min="7" max="7" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="36.5703125" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="37.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" customWidth="1"/>
+    <col min="5" max="5" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="36.5546875" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1184,729 +1690,1076 @@
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="16">
+        <v>26</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="15">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="10"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
+      <c r="C2" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="15">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D3" s="4"/>
+      <c r="C3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="3"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="16">
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="15">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="2"/>
+      <c r="C4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="16">
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="15">
         <v>9</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="4"/>
+      <c r="B5" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>98</v>
+      </c>
       <c r="D5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="2"/>
+      <c r="E5" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="15">
         <v>7</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="12"/>
+      <c r="C6" s="21" t="s">
+        <v>102</v>
+      </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="15">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="4"/>
+      <c r="B7" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>115</v>
+      </c>
       <c r="D7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="E7" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="16">
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="15">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="12"/>
+      <c r="C8" s="11" t="s">
+        <v>116</v>
+      </c>
       <c r="D8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="7" t="s">
-        <v>77</v>
+      <c r="H8" s="6" t="s">
+        <v>76</v>
       </c>
       <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="15">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="4"/>
+      <c r="B9" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="D9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="16">
+      <c r="E9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="15">
         <v>2</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="16">
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="15">
         <v>1</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>42</v>
+      <c r="C11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="16">
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="15">
         <v>3</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="18" t="s">
+      <c r="F12" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="G12" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2" t="s">
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="15">
+        <v>2</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="16">
-        <v>2</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="D13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="15">
+        <v>1</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="15">
+        <v>1</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="3"/>
+      <c r="E15" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="16">
+      <c r="F15" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15">
         <v>1</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
+      <c r="B16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="13"/>
+      <c r="E16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="15">
         <v>1</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="2"/>
-    </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16">
-        <v>1</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H16" s="7"/>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16">
-        <v>1</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
+      <c r="B17" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="11"/>
+      <c r="F17" s="10"/>
       <c r="G17" s="2"/>
-      <c r="H17" s="7"/>
+      <c r="H17" s="6"/>
       <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="16">
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="15">
         <v>3</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="B18" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="15">
         <v>1</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
+      <c r="B19" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="11"/>
+      <c r="F19" s="10"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="16">
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="15">
         <v>1</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
+      <c r="B20" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="11"/>
+      <c r="F20" s="10"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="16">
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="15">
         <v>1</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="3"/>
+      <c r="E21" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="F21" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="16">
+        <v>61</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="15">
         <v>1</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="C22" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>129</v>
+      </c>
       <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
+      <c r="I22" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J22" s="25" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="15">
         <v>1</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
       <c r="H23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="16">
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="15">
         <v>1</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="16">
+      <c r="C24" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="15">
+        <v>12</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="15">
+        <v>2</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="15">
         <v>1</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-    </row>
-    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="16">
-        <v>12</v>
-      </c>
-      <c r="B26" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="16">
-        <v>2</v>
-      </c>
-      <c r="B27" s="4" t="s">
+      <c r="C27" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="15">
+        <v>1</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="15">
+        <v>5</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="G29" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="15">
+        <v>1</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="16">
-        <v>1</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="16">
-        <v>1</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="16">
-        <v>5</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="2"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="16">
-        <v>1</v>
-      </c>
-      <c r="B31" s="4" t="s">
+      <c r="C30" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="15">
+        <v>4</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
+      <c r="C31" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>167</v>
+      </c>
       <c r="I31" s="2"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="16">
-        <v>4</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
+      <c r="J31" s="2"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="15">
+        <v>11</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
+      <c r="G32" s="3"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="16">
-        <v>11</v>
-      </c>
-      <c r="B33" s="4" t="s">
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="15">
+        <v>1</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="16">
+      <c r="C33" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>175</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="J33" s="2"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="15">
         <v>1</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="16">
+      <c r="C34" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D34" s="30" t="s">
+        <v>181</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="J34" s="2"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="15">
         <v>1</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="16">
+      <c r="C35" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D35" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J35" s="2"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="15">
         <v>1</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="16">
+      <c r="C36" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D36" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I36" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="J36" s="2"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="15">
         <v>1</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C37" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="J37" s="2"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="16">
         <v>1</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="11"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="17">
+      <c r="C38" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="D38" s="30" t="s">
+        <v>208</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="I38" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="J38" s="2"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" s="16">
         <v>1</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="B39" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="17">
+      <c r="C39" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D39" s="30" t="s">
+        <v>215</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="I39" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="J39" s="2"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" s="16">
         <v>1</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="11"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="17">
-        <v>1</v>
-      </c>
-      <c r="B41" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="11"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="15">
-        <f>SUM(A2:A41)</f>
-        <v>93</v>
-      </c>
-      <c r="B42" s="9" t="s">
+      <c r="C40" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="I40" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="J40" s="10"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" s="14">
+        <f>SUM(A2:A40)</f>
+        <v>92</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" display="https://www.digikey.com/en/products/detail/taoglas-limited/SGGP-25-2-A-02/6362788?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=17922795960&amp;gbraid=0AAAAADrbLlgMcI_xxgM1XnWlukN8LfDyD&amp;gclid=Cj0KCQjwl5jHBhDHARIsAB0YqjwtykcaCqflOK956I59n-BT9VoB2bK0Yaz9wxJRDuOLV2NKlyDRbr8aAiUgEALw_wcB" xr:uid="{EAA79944-4731-42F6-A8F3-A9938CAA121C}"/>
+    <hyperlink ref="F22" r:id="rId2" display="https://www.mouser.com/manufacturer/coilcraft/" xr:uid="{CED89B1A-921B-483C-94A5-D3D0D17FB929}"/>
+    <hyperlink ref="D22" r:id="rId3" display="https://www.mouser.com/c/passive-components/inductors-chokes-coils/power-inductors-smd/?m=Coilcraft&amp;series=LPS3010" xr:uid="{8A83DDD0-1C33-4EDB-A035-13D20D09AE17}"/>
+    <hyperlink ref="D24" r:id="rId4" display="https://www.digikey.com/en/products/filter/transistors/fets-mosfets/single-fets-mosfets/to-236-3-sc-59-sot-23-3/278?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQA3AOygBcAnAV3xAHsoBtEAFjAGZ2wAOEAXQIAHMlBABlSgEtiAcxABfRUA" xr:uid="{FD328100-F3B7-4B69-B0ED-4FAB1791735F}"/>
+    <hyperlink ref="D30" r:id="rId5" display="https://www.digikey.com/en/products/result?s=N4IgjCBcoLQCxVAYygMwIYBsDOBTANCAG4B2aWehA9lANohwAccAzAEwgC6hADgC5QQIAL6igA" xr:uid="{C81535BB-A5C7-4FDD-B4D2-90F7FB1E8938}"/>
+    <hyperlink ref="D31" r:id="rId6" display="https://www.digikey.com/en/products/result?s=N4IgjCBcoLQCxVAYygMwIYBsDOBTANCAG4B2aWehA9lANogCcArHEwGwgC6hADgC5QQIAL6igA" xr:uid="{FF71EE82-24FA-4A30-A704-B40120AE9746}"/>
+    <hyperlink ref="D35" r:id="rId7" display="https://www.digikey.com/en/products/filter/power-management-pmic/voltage-regulators-dc-dc-switching-regulators/10-wfdfn-exposed-pad/739?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQA3AOygBcAnAV3xAHsoBtEAdgBZ2BOEAXQIAcyUEAGVKAS2IBzEAF95QA" xr:uid="{08D2A1B0-FCC3-46BD-AA04-BBCD507C76C4}"/>
+    <hyperlink ref="I36" r:id="rId8" xr:uid="{504861C4-2BAC-4BE2-8F95-7EA09BF4415C}"/>
+    <hyperlink ref="I38" r:id="rId9" xr:uid="{BB78B275-38B4-4555-BEEE-09680AD6EE69}"/>
+    <hyperlink ref="I39" r:id="rId10" xr:uid="{4295295F-C461-46B4-9FF8-784C0631F89D}"/>
+  </hyperlinks>
   <pageMargins left="0.67965686274509796" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="59" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="59" orientation="landscape" r:id="rId11"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"-,Bold"&amp;14Golf GPS BOM&amp;RRev 1</oddHeader>
   </headerFooter>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BOM work can be overwritten
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\gitRepos\golf-gps\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1eb1c9bb38a56ae9/Documents/CollegeInformation/2025-2026/EE333/golf-gps/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341176FB-9001-4A4D-A907-A9F20D64AA81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{341176FB-9001-4A4D-A907-A9F20D64AA81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBC79DE7-0BE6-4AB0-83CB-CB96545B6C14}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -833,7 +833,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -858,15 +858,124 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+        <bottom style="thin">
+          <color theme="9"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="9"/>
+        </left>
         <right style="thin">
           <color theme="9"/>
         </right>
@@ -897,11 +1006,9 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
+        <left/>
         <right style="thin">
           <color theme="9"/>
         </right>
@@ -914,12 +1021,20 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border>
+        <top style="thin">
+          <color theme="9"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color theme="9"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color theme="9"/>
+        </right>
         <top style="thin">
           <color theme="9"/>
         </top>
@@ -929,85 +1044,7 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
+      <border>
         <bottom style="thin">
           <color theme="9"/>
         </bottom>
@@ -1029,36 +1066,6 @@
         <horizontal style="thin">
           <color theme="9"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="9"/>
-        </left>
-        <right style="thin">
-          <color theme="9"/>
-        </right>
-        <top style="thin">
-          <color theme="9"/>
-        </top>
-        <bottom style="thin">
-          <color theme="9"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
@@ -1075,7 +1082,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:I39" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}" name="Table2" displayName="Table2" ref="A1:I39" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="A1:I39" xr:uid="{D97A74AA-1858-4C6A-B21B-3D6DECA4386F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1088,15 +1095,15 @@
     <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{32AFDCD7-F4DF-4ED5-8811-A4897B942137}" name="Quantity" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{FE933B93-DA18-4AED-A480-8EB2CB37E9FA}" name="Reference(s)" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{F7578A95-5131-4E48-843B-E8DF71CB7A4C}" name="Description" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{0E106ADB-04B7-4862-9B8C-0C8A8ACABA2E}" name="Package" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{3756D777-6A0B-46EA-891A-5F8ACDDB5DC3}" name="Part Number" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{E9BD92E7-ABBB-4AE0-9D4B-0267526E38F6}" name="Manufacturer" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{F268DED4-AA10-4CEF-A3B9-66A35E6F6B34}" name="Vendor PN" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{123ECB15-FDBD-41FB-B610-A68574792B2E}" name="Notes" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{CBC1BA7D-9405-443F-AA6B-33103FF6355C}" name="Link" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1366,20 +1373,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="37.6640625" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.42578125" customWidth="1"/>
-    <col min="9" max="9" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.44140625" customWidth="1"/>
+    <col min="9" max="9" width="255.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1408,7 +1415,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -1433,7 +1440,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <v>1</v>
       </c>
@@ -1458,7 +1465,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -1483,7 +1490,7 @@
       </c>
       <c r="I4" s="7"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>7</v>
       </c>
@@ -1510,7 +1517,7 @@
       </c>
       <c r="I5" s="7"/>
     </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>8</v>
       </c>
@@ -1537,7 +1544,7 @@
       </c>
       <c r="I6" s="7"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>2</v>
       </c>
@@ -1564,7 +1571,7 @@
       </c>
       <c r="I7" s="7"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>2</v>
       </c>
@@ -1589,7 +1596,7 @@
       <c r="H8" s="6"/>
       <c r="I8" s="7"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <v>3</v>
       </c>
@@ -1614,7 +1621,7 @@
       <c r="H9" s="6"/>
       <c r="I9" s="7"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="12">
         <v>1</v>
       </c>
@@ -1639,7 +1646,7 @@
       <c r="H10" s="6"/>
       <c r="I10" s="7"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
         <v>2</v>
       </c>
@@ -1666,7 +1673,7 @@
       </c>
       <c r="I11" s="7"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
         <v>1</v>
       </c>
@@ -1693,7 +1700,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="12">
         <v>1</v>
       </c>
@@ -1718,7 +1725,7 @@
       <c r="H13" s="6"/>
       <c r="I13" s="7"/>
     </row>
-    <row r="14" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="12">
         <v>1</v>
       </c>
@@ -1743,7 +1750,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12">
         <v>1</v>
       </c>
@@ -1764,7 +1771,7 @@
       </c>
       <c r="I15" s="7"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="12">
         <v>1</v>
       </c>
@@ -1785,7 +1792,7 @@
       </c>
       <c r="I16" s="7"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="12">
         <v>1</v>
       </c>
@@ -1806,7 +1813,7 @@
       </c>
       <c r="I17" s="7"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="12">
         <v>1</v>
       </c>
@@ -1827,7 +1834,7 @@
       </c>
       <c r="I18" s="7"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="12">
         <v>1</v>
       </c>
@@ -1854,7 +1861,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="12">
         <v>1</v>
       </c>
@@ -1877,7 +1884,7 @@
       <c r="H20" s="6"/>
       <c r="I20" s="7"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="12">
         <v>1</v>
       </c>
@@ -1894,7 +1901,7 @@
       </c>
       <c r="I21" s="7"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="12">
         <v>1</v>
       </c>
@@ -1921,7 +1928,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="12">
         <v>2</v>
       </c>
@@ -1948,7 +1955,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="12">
         <v>1</v>
       </c>
@@ -1975,7 +1982,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="12">
         <v>8</v>
       </c>
@@ -2002,7 +2009,7 @@
       </c>
       <c r="I25" s="7"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="12">
         <v>5</v>
       </c>
@@ -2029,7 +2036,7 @@
       </c>
       <c r="I26" s="7"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="12">
         <v>2</v>
       </c>
@@ -2054,14 +2061,14 @@
       <c r="H27" s="6"/>
       <c r="I27" s="7"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
-        <v>1</v>
-      </c>
-      <c r="B28" s="10" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="14">
+        <v>1</v>
+      </c>
+      <c r="B28" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="16" t="s">
         <v>196</v>
       </c>
       <c r="D28" s="6" t="s">
@@ -2081,14 +2088,14 @@
       </c>
       <c r="I28" s="7"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="12">
-        <v>1</v>
-      </c>
-      <c r="B29" s="10" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="14">
+        <v>1</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="16" t="s">
         <v>199</v>
       </c>
       <c r="D29" s="6" t="s">
@@ -2106,14 +2113,14 @@
       <c r="H29" s="6"/>
       <c r="I29" s="7"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="12">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="14">
         <v>2</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="16" t="s">
         <v>204</v>
       </c>
       <c r="D30" s="6" t="s">
@@ -2131,7 +2138,7 @@
       <c r="H30" s="6"/>
       <c r="I30" s="7"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="12">
         <v>1</v>
       </c>
@@ -2156,7 +2163,7 @@
       </c>
       <c r="I31" s="7"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="12">
         <v>4</v>
       </c>
@@ -2175,7 +2182,7 @@
       </c>
       <c r="I32" s="7"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="12">
         <v>1</v>
       </c>
@@ -2202,7 +2209,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="12">
         <v>1</v>
       </c>
@@ -2229,7 +2236,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="12">
         <v>1</v>
       </c>
@@ -2256,7 +2263,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="12">
         <v>1</v>
       </c>
@@ -2283,7 +2290,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="12">
         <v>1</v>
       </c>
@@ -2310,7 +2317,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="12">
         <v>1</v>
       </c>
@@ -2337,7 +2344,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="13">
         <v>1</v>
       </c>
@@ -2364,7 +2371,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <f>SUM(A2:A39)</f>
         <v>73</v>

</xml_diff>

<commit_message>
Started hardware test program. Found required libraries
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\gitRepos\golf-gps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5FB8036-24B6-4115-8B42-5F18822F7FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EB08B9-4EE8-41D7-B177-4903B3089780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="208">
   <si>
     <t>Quantity</t>
   </si>
@@ -660,6 +660,22 @@
   </si>
   <si>
     <t>TE Connectivity</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ETG Stock, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DNP R12, R13</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1989,7 +2005,7 @@
         <v>86</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>38</v>
+        <v>207</v>
       </c>
       <c r="I25" s="7"/>
     </row>

</xml_diff>

<commit_message>
Added new OLED footprint. Finished schematic updates, started lyout. Changed 10 mOhm sense resistor PN to TCR of 50 ppm/C
</commit_message>
<xml_diff>
--- a/docs/BOM.xlsx
+++ b/docs/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\gitRepos\golf-gps\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bjkuh\Projects\gitRepos\golf-gps\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5FB8036-24B6-4115-8B42-5F18822F7FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C698859-7009-4E8F-9471-A767F12B9553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28695" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="208">
   <si>
     <t>Quantity</t>
   </si>
@@ -605,9 +605,6 @@
     <t>IC FUEL GAUGE LI-ION 1CELL 12SON</t>
   </si>
   <si>
-    <t>1% tolerance, 1W rating</t>
-  </si>
-  <si>
     <t>1206</t>
   </si>
   <si>
@@ -629,12 +626,6 @@
     <t>RES 0.01 OHM 1% 1W 1206</t>
   </si>
   <si>
-    <t>CSRF1206FT10L0</t>
-  </si>
-  <si>
-    <t>CSRF1206FT10L0CT-ND</t>
-  </si>
-  <si>
     <t>RES 470K OHM 5% 1/8W 0805</t>
   </si>
   <si>
@@ -660,6 +651,18 @@
   </si>
   <si>
     <t>TE Connectivity</t>
+  </si>
+  <si>
+    <t>MCP73871-1AAI/ML</t>
+  </si>
+  <si>
+    <t>1% tolerance, 1W rating, 50ppm TCR</t>
+  </si>
+  <si>
+    <t>CSNL1206FT10L0</t>
+  </si>
+  <si>
+    <t>CSNL1206FT10L0CT-ND</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1365,7 @@
     <col min="5" max="5" width="28.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.42578125" customWidth="1"/>
+    <col min="8" max="8" width="33.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1691,7 +1694,7 @@
         <v>50</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>47</v>
@@ -1741,16 +1744,16 @@
         <v>152</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>38</v>
@@ -1768,7 +1771,7 @@
         <v>172</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
@@ -1789,7 +1792,7 @@
         <v>176</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
@@ -1810,7 +1813,7 @@
         <v>175</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -2034,13 +2037,13 @@
         <v>83</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>85</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H27" s="6"/>
       <c r="I27" s="7"/>
@@ -2053,22 +2056,22 @@
         <v>182</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>85</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>188</v>
+        <v>205</v>
       </c>
       <c r="I28" s="7"/>
     </row>
@@ -2080,19 +2083,19 @@
         <v>183</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>85</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H29" s="6"/>
       <c r="I29" s="7"/>
@@ -2105,19 +2108,19 @@
         <v>184</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>85</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H30" s="6"/>
       <c r="I30" s="7"/>
@@ -2132,7 +2135,9 @@
       <c r="C31" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D31" s="6"/>
+      <c r="D31" s="6" t="s">
+        <v>189</v>
+      </c>
       <c r="E31" s="6" t="s">
         <v>141</v>
       </c>
@@ -2180,7 +2185,7 @@
         <v>146</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>112</v>
+        <v>204</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>111</v>

</xml_diff>